<commit_message>
Updated following scripts and added GAMESSUS calculator. oled_energy_calc, organic_phos_calc to use TBLite and GAMESSUS calculators
</commit_message>
<xml_diff>
--- a/organic_phos.xlsx
+++ b/organic_phos.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/zhuan08/Programming Projects/oled-project/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/zhuan08/Programming_Projects/oled_project/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0EC3A055-315D-0143-92E7-11A5D6F5A28C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{747DFFA5-1A03-1248-B70F-EA294265C219}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="740" windowWidth="29400" windowHeight="17000" xr2:uid="{DF7F3765-FD89-0D40-8244-227DDC256222}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="20" uniqueCount="20">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="29" uniqueCount="22">
   <si>
     <t>predicted</t>
   </si>
@@ -96,6 +96,12 @@
   </si>
   <si>
     <t>Brc1ccc(-c2ccc(Br)cc2)cc1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">dcbp </t>
+  </si>
+  <si>
+    <t>tblie geom w/ gamess calc</t>
   </si>
 </sst>
 </file>
@@ -206,26 +212,6 @@
         </a:ln>
         <a:effectLst/>
       </c:spPr>
-      <c:txPr>
-        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
-        <a:lstStyle/>
-        <a:p>
-          <a:pPr>
-            <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
-              <a:solidFill>
-                <a:schemeClr val="tx1">
-                  <a:lumMod val="65000"/>
-                  <a:lumOff val="35000"/>
-                </a:schemeClr>
-              </a:solidFill>
-              <a:latin typeface="+mn-lt"/>
-              <a:ea typeface="+mn-ea"/>
-              <a:cs typeface="+mn-cs"/>
-            </a:defRPr>
-          </a:pPr>
-          <a:endParaRPr lang="en-US"/>
-        </a:p>
-      </c:txPr>
     </c:title>
     <c:autoTitleDeleted val="0"/>
     <c:plotArea>
@@ -234,8 +220,92 @@
         <c:scatterStyle val="lineMarker"/>
         <c:varyColors val="0"/>
         <c:ser>
+          <c:idx val="1"/>
+          <c:order val="0"/>
+          <c:tx>
+            <c:v>predicted</c:v>
+          </c:tx>
+          <c:spPr>
+            <a:ln w="38100">
+              <a:noFill/>
+            </a:ln>
+          </c:spPr>
+          <c:xVal>
+            <c:numRef>
+              <c:f>Sheet1!$C$2:$C$9</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="8"/>
+                <c:pt idx="0">
+                  <c:v>2.9520047246000001</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>3.0313984946992698</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>2.94499283689311</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>2.8968270661962601</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>2.94499283689311</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>2.58839662699791</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>3.6681715512781099</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>2.5830041340249998</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:xVal>
+          <c:yVal>
+            <c:numRef>
+              <c:f>Sheet1!$D$2:$D$9</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="8"/>
+                <c:pt idx="0">
+                  <c:v>2.6503877528168598</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>2.6649325265323101</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>2.5977483063393199</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>2.54076374062651</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>2.5876237612164901</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>1.83320161865776</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>3.09235839203461</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>2.4915844109666501</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:yVal>
+          <c:smooth val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{0000000C-11ED-3C43-B1C3-C422CD39C77E}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:ser>
           <c:idx val="0"/>
-          <c:order val="0"/>
+          <c:order val="1"/>
           <c:tx>
             <c:v>predicted</c:v>
           </c:tx>
@@ -275,7 +345,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{5B9DEAA0-A5E8-5B49-ACE8-D4760ACE85E7}" type="CELLRANGE">
+                    <a:fld id="{B0C3F812-59C0-554D-814C-17E39E884EF1}" type="CELLRANGE">
                       <a:rPr lang="en-US"/>
                       <a:pPr/>
                       <a:t>[CELLRANGE]</a:t>
@@ -297,7 +367,7 @@
                   <c15:showDataLabelsRange val="1"/>
                 </c:ext>
                 <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-                  <c16:uniqueId val="{00000003-BFD8-5241-B121-31D681B22365}"/>
+                  <c16:uniqueId val="{00000002-11ED-3C43-B1C3-C422CD39C77E}"/>
                 </c:ext>
               </c:extLst>
             </c:dLbl>
@@ -314,7 +384,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{98628232-B2E2-4049-8A9C-F83DABF06D53}" type="CELLRANGE">
+                    <a:fld id="{495833C4-83E9-EA4A-8301-1093E39B44ED}" type="CELLRANGE">
                       <a:rPr lang="en-US"/>
                       <a:pPr/>
                       <a:t>[CELLRANGE]</a:t>
@@ -336,7 +406,7 @@
                   <c15:showDataLabelsRange val="1"/>
                 </c:ext>
                 <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-                  <c16:uniqueId val="{00000004-BFD8-5241-B121-31D681B22365}"/>
+                  <c16:uniqueId val="{00000003-11ED-3C43-B1C3-C422CD39C77E}"/>
                 </c:ext>
               </c:extLst>
             </c:dLbl>
@@ -353,7 +423,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{027E1E81-108E-4748-84C7-D7A130E65344}" type="CELLRANGE">
+                    <a:fld id="{76C40F15-E9B0-F34C-862C-4B374E217320}" type="CELLRANGE">
                       <a:rPr lang="en-US"/>
                       <a:pPr/>
                       <a:t>[CELLRANGE]</a:t>
@@ -375,7 +445,7 @@
                   <c15:showDataLabelsRange val="1"/>
                 </c:ext>
                 <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-                  <c16:uniqueId val="{00000005-BFD8-5241-B121-31D681B22365}"/>
+                  <c16:uniqueId val="{00000004-11ED-3C43-B1C3-C422CD39C77E}"/>
                 </c:ext>
               </c:extLst>
             </c:dLbl>
@@ -392,7 +462,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{0122BDCE-EB46-E34E-8077-4C15A43B4F3E}" type="CELLRANGE">
+                    <a:fld id="{0F822F01-5873-CA4D-9E88-F1F0D567504E}" type="CELLRANGE">
                       <a:rPr lang="en-US"/>
                       <a:pPr/>
                       <a:t>[CELLRANGE]</a:t>
@@ -414,7 +484,7 @@
                   <c15:showDataLabelsRange val="1"/>
                 </c:ext>
                 <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-                  <c16:uniqueId val="{00000006-BFD8-5241-B121-31D681B22365}"/>
+                  <c16:uniqueId val="{00000005-11ED-3C43-B1C3-C422CD39C77E}"/>
                 </c:ext>
               </c:extLst>
             </c:dLbl>
@@ -431,7 +501,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{FE845039-0FDE-004E-972C-5B19D5B7189D}" type="CELLRANGE">
+                    <a:fld id="{A28D18E8-6E38-5F49-A0C6-F3A983D5CFDB}" type="CELLRANGE">
                       <a:rPr lang="en-US"/>
                       <a:pPr/>
                       <a:t>[CELLRANGE]</a:t>
@@ -453,7 +523,7 @@
                   <c15:showDataLabelsRange val="1"/>
                 </c:ext>
                 <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-                  <c16:uniqueId val="{00000007-BFD8-5241-B121-31D681B22365}"/>
+                  <c16:uniqueId val="{00000006-11ED-3C43-B1C3-C422CD39C77E}"/>
                 </c:ext>
               </c:extLst>
             </c:dLbl>
@@ -470,7 +540,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{76BFEC26-94D7-7A47-8F6D-2FF9F045A6FB}" type="CELLRANGE">
+                    <a:fld id="{EC79FEDB-C104-4C48-B0BF-4B606D21591C}" type="CELLRANGE">
                       <a:rPr lang="en-US"/>
                       <a:pPr/>
                       <a:t>[CELLRANGE]</a:t>
@@ -492,7 +562,7 @@
                   <c15:showDataLabelsRange val="1"/>
                 </c:ext>
                 <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-                  <c16:uniqueId val="{00000008-BFD8-5241-B121-31D681B22365}"/>
+                  <c16:uniqueId val="{00000007-11ED-3C43-B1C3-C422CD39C77E}"/>
                 </c:ext>
               </c:extLst>
             </c:dLbl>
@@ -509,7 +579,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{F09E4D15-71ED-6640-8FC6-ABA5CE293BD5}" type="CELLRANGE">
+                    <a:fld id="{E3789AD0-37CB-BC4F-9D0C-67D07E9A6978}" type="CELLRANGE">
                       <a:rPr lang="en-US"/>
                       <a:pPr/>
                       <a:t>[CELLRANGE]</a:t>
@@ -531,7 +601,7 @@
                   <c15:showDataLabelsRange val="1"/>
                 </c:ext>
                 <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-                  <c16:uniqueId val="{00000002-BFD8-5241-B121-31D681B22365}"/>
+                  <c16:uniqueId val="{00000008-11ED-3C43-B1C3-C422CD39C77E}"/>
                 </c:ext>
               </c:extLst>
             </c:dLbl>
@@ -548,7 +618,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{87B2E46D-C75E-2B40-B372-AB8282779BC1}" type="CELLRANGE">
+                    <a:fld id="{FA78989F-5AEF-FA44-A58E-E8423DBD5C48}" type="CELLRANGE">
                       <a:rPr lang="en-US"/>
                       <a:pPr/>
                       <a:t>[CELLRANGE]</a:t>
@@ -570,7 +640,7 @@
                   <c15:showDataLabelsRange val="1"/>
                 </c:ext>
                 <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-                  <c16:uniqueId val="{00000009-BFD8-5241-B121-31D681B22365}"/>
+                  <c16:uniqueId val="{00000009-11ED-3C43-B1C3-C422CD39C77E}"/>
                 </c:ext>
               </c:extLst>
             </c:dLbl>
@@ -783,7 +853,7 @@
               </c15:datalabelsRange>
             </c:ext>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000000-BFD8-5241-B121-31D681B22365}"/>
+              <c16:uniqueId val="{0000000B-11ED-3C43-B1C3-C422CD39C77E}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -841,26 +911,6 @@
             </a:ln>
             <a:effectLst/>
           </c:spPr>
-          <c:txPr>
-            <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
-            <a:lstStyle/>
-            <a:p>
-              <a:pPr>
-                <a:defRPr sz="1000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
-                  <a:solidFill>
-                    <a:schemeClr val="tx1">
-                      <a:lumMod val="65000"/>
-                      <a:lumOff val="35000"/>
-                    </a:schemeClr>
-                  </a:solidFill>
-                  <a:latin typeface="+mn-lt"/>
-                  <a:ea typeface="+mn-ea"/>
-                  <a:cs typeface="+mn-cs"/>
-                </a:defRPr>
-              </a:pPr>
-              <a:endParaRPr lang="en-US"/>
-            </a:p>
-          </c:txPr>
         </c:title>
         <c:numFmt formatCode="General" sourceLinked="1"/>
         <c:majorTickMark val="none"/>
@@ -946,26 +996,6 @@
             </a:ln>
             <a:effectLst/>
           </c:spPr>
-          <c:txPr>
-            <a:bodyPr rot="-5400000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
-            <a:lstStyle/>
-            <a:p>
-              <a:pPr>
-                <a:defRPr sz="1000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
-                  <a:solidFill>
-                    <a:schemeClr val="tx1">
-                      <a:lumMod val="65000"/>
-                      <a:lumOff val="35000"/>
-                    </a:schemeClr>
-                  </a:solidFill>
-                  <a:latin typeface="+mn-lt"/>
-                  <a:ea typeface="+mn-ea"/>
-                  <a:cs typeface="+mn-cs"/>
-                </a:defRPr>
-              </a:pPr>
-              <a:endParaRPr lang="en-US"/>
-            </a:p>
-          </c:txPr>
         </c:title>
         <c:numFmt formatCode="General" sourceLinked="1"/>
         <c:majorTickMark val="none"/>
@@ -1047,6 +1077,480 @@
         </a:p>
       </c:txPr>
     </c:legend>
+    <c:plotVisOnly val="1"/>
+    <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
+    <c:extLst/>
+  </c:chart>
+  <c:txPr>
+    <a:bodyPr/>
+    <a:lstStyle/>
+    <a:p>
+      <a:pPr>
+        <a:defRPr/>
+      </a:pPr>
+      <a:endParaRPr lang="en-US"/>
+    </a:p>
+  </c:txPr>
+  <c:printSettings>
+    <c:headerFooter/>
+    <c:pageMargins b="0.75" l="0.7" r="0.7" t="0.75" header="0.3" footer="0.3"/>
+    <c:pageSetup/>
+  </c:printSettings>
+</c:chartSpace>
+</file>
+
+<file path=xl/charts/chart2.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
+  <c:date1904 val="0"/>
+  <c:lang val="en-US"/>
+  <c:roundedCorners val="0"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
+      <c14:style val="102"/>
+    </mc:Choice>
+    <mc:Fallback>
+      <c:style val="2"/>
+    </mc:Fallback>
+  </mc:AlternateContent>
+  <c:chart>
+    <c:title>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="65000"/>
+                  <a:lumOff val="35000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr lang="en-US"/>
+        </a:p>
+      </c:txPr>
+    </c:title>
+    <c:autoTitleDeleted val="0"/>
+    <c:plotArea>
+      <c:layout/>
+      <c:scatterChart>
+        <c:scatterStyle val="lineMarker"/>
+        <c:varyColors val="0"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:spPr>
+            <a:ln w="38100" cap="rnd">
+              <a:noFill/>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="circle"/>
+            <c:size val="5"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent1"/>
+              </a:solidFill>
+              <a:ln w="9525">
+                <a:solidFill>
+                  <a:schemeClr val="accent1"/>
+                </a:solidFill>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+          </c:marker>
+          <c:trendline>
+            <c:spPr>
+              <a:ln w="19050" cap="rnd">
+                <a:solidFill>
+                  <a:schemeClr val="accent1"/>
+                </a:solidFill>
+                <a:prstDash val="sysDot"/>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+            <c:trendlineType val="linear"/>
+            <c:dispRSqr val="1"/>
+            <c:dispEq val="1"/>
+            <c:trendlineLbl>
+              <c:layout>
+                <c:manualLayout>
+                  <c:x val="-0.30051509186351705"/>
+                  <c:y val="-0.11150991542723826"/>
+                </c:manualLayout>
+              </c:layout>
+              <c:numFmt formatCode="General" sourceLinked="0"/>
+              <c:spPr>
+                <a:noFill/>
+                <a:ln>
+                  <a:noFill/>
+                </a:ln>
+                <a:effectLst/>
+              </c:spPr>
+              <c:txPr>
+                <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+                <a:lstStyle/>
+                <a:p>
+                  <a:pPr>
+                    <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                      <a:solidFill>
+                        <a:schemeClr val="tx1">
+                          <a:lumMod val="65000"/>
+                          <a:lumOff val="35000"/>
+                        </a:schemeClr>
+                      </a:solidFill>
+                      <a:latin typeface="+mn-lt"/>
+                      <a:ea typeface="+mn-ea"/>
+                      <a:cs typeface="+mn-cs"/>
+                    </a:defRPr>
+                  </a:pPr>
+                  <a:endParaRPr lang="en-US"/>
+                </a:p>
+              </c:txPr>
+            </c:trendlineLbl>
+          </c:trendline>
+          <c:xVal>
+            <c:numRef>
+              <c:f>Sheet1!$C$2:$C$9</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="8"/>
+                <c:pt idx="0">
+                  <c:v>2.9520047246000001</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>3.0313984946992698</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>2.94499283689311</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>2.8968270661962601</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>2.94499283689311</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>2.58839662699791</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>3.6681715512781099</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>2.5830041340249998</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:xVal>
+          <c:yVal>
+            <c:numRef>
+              <c:f>Sheet1!$G$2:$G$9</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="8"/>
+                <c:pt idx="0">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>1.41730194714546</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>1.4176127011742199</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>1.2780348272281099</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>0.88988790262010298</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>2.7341953492741502</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>1.4755046936425</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:yVal>
+          <c:smooth val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000000-A1B9-0643-A068-5B68B356BEC9}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:dLbls>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="0"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+        </c:dLbls>
+        <c:axId val="1253394272"/>
+        <c:axId val="376033183"/>
+      </c:scatterChart>
+      <c:valAx>
+        <c:axId val="1253394272"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="b"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="15000"/>
+                  <a:lumOff val="85000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:title>
+          <c:tx>
+            <c:rich>
+              <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr sz="1000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                    <a:solidFill>
+                      <a:schemeClr val="tx1">
+                        <a:lumMod val="65000"/>
+                        <a:lumOff val="35000"/>
+                      </a:schemeClr>
+                    </a:solidFill>
+                    <a:latin typeface="+mn-lt"/>
+                    <a:ea typeface="+mn-ea"/>
+                    <a:cs typeface="+mn-cs"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:r>
+                  <a:rPr lang="en-US"/>
+                  <a:t>actual</a:t>
+                </a:r>
+              </a:p>
+            </c:rich>
+          </c:tx>
+          <c:overlay val="0"/>
+          <c:spPr>
+            <a:noFill/>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:txPr>
+            <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+            <a:lstStyle/>
+            <a:p>
+              <a:pPr>
+                <a:defRPr sz="1000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                  <a:solidFill>
+                    <a:schemeClr val="tx1">
+                      <a:lumMod val="65000"/>
+                      <a:lumOff val="35000"/>
+                    </a:schemeClr>
+                  </a:solidFill>
+                  <a:latin typeface="+mn-lt"/>
+                  <a:ea typeface="+mn-ea"/>
+                  <a:cs typeface="+mn-cs"/>
+                </a:defRPr>
+              </a:pPr>
+              <a:endParaRPr lang="en-US"/>
+            </a:p>
+          </c:txPr>
+        </c:title>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+            <a:solidFill>
+              <a:schemeClr val="tx1">
+                <a:lumMod val="25000"/>
+                <a:lumOff val="75000"/>
+              </a:schemeClr>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="en-US"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="376033183"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="midCat"/>
+      </c:valAx>
+      <c:valAx>
+        <c:axId val="376033183"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="l"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="15000"/>
+                  <a:lumOff val="85000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:title>
+          <c:tx>
+            <c:rich>
+              <a:bodyPr rot="-5400000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr sz="1000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                    <a:solidFill>
+                      <a:schemeClr val="tx1">
+                        <a:lumMod val="65000"/>
+                        <a:lumOff val="35000"/>
+                      </a:schemeClr>
+                    </a:solidFill>
+                    <a:latin typeface="+mn-lt"/>
+                    <a:ea typeface="+mn-ea"/>
+                    <a:cs typeface="+mn-cs"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:r>
+                  <a:rPr lang="en-US"/>
+                  <a:t>predict</a:t>
+                </a:r>
+              </a:p>
+            </c:rich>
+          </c:tx>
+          <c:overlay val="0"/>
+          <c:spPr>
+            <a:noFill/>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:txPr>
+            <a:bodyPr rot="-5400000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+            <a:lstStyle/>
+            <a:p>
+              <a:pPr>
+                <a:defRPr sz="1000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                  <a:solidFill>
+                    <a:schemeClr val="tx1">
+                      <a:lumMod val="65000"/>
+                      <a:lumOff val="35000"/>
+                    </a:schemeClr>
+                  </a:solidFill>
+                  <a:latin typeface="+mn-lt"/>
+                  <a:ea typeface="+mn-ea"/>
+                  <a:cs typeface="+mn-cs"/>
+                </a:defRPr>
+              </a:pPr>
+              <a:endParaRPr lang="en-US"/>
+            </a:p>
+          </c:txPr>
+        </c:title>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+            <a:solidFill>
+              <a:schemeClr val="tx1">
+                <a:lumMod val="25000"/>
+                <a:lumOff val="75000"/>
+              </a:schemeClr>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="en-US"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="1253394272"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="midCat"/>
+      </c:valAx>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+    </c:plotArea>
     <c:plotVisOnly val="1"/>
     <c:dispBlanksAs val="gap"/>
     <c:extLst>
@@ -1680,6 +2184,42 @@
       <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
           <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>5</xdr:col>
+      <xdr:colOff>508000</xdr:colOff>
+      <xdr:row>12</xdr:row>
+      <xdr:rowOff>172720</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>10</xdr:col>
+      <xdr:colOff>254000</xdr:colOff>
+      <xdr:row>26</xdr:row>
+      <xdr:rowOff>71120</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame macro="">
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="3" name="Chart 2">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{937F125C-BCF2-63B4-974C-CFA18222B666}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvGraphicFramePr/>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="0" y="0"/>
+        <a:ext cx="0" cy="0"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId2"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -2005,7 +2545,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{437ED259-CF5A-CE41-806D-66384DA86059}">
-  <dimension ref="A1:D9"/>
+  <dimension ref="A1:G9"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="6.5" bestFit="1" customWidth="1"/>
@@ -2013,9 +2553,10 @@
     <col min="3" max="3" width="14.5" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="12.6640625" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="12.1640625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="20.1640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>1</v>
       </c>
@@ -2028,8 +2569,11 @@
       <c r="D1" s="1" t="s">
         <v>0</v>
       </c>
+      <c r="F1" s="1" t="s">
+        <v>21</v>
+      </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A2" s="1" t="s">
         <v>4</v>
       </c>
@@ -2042,8 +2586,14 @@
       <c r="D2">
         <v>2.6503877528168598</v>
       </c>
+      <c r="F2" t="s">
+        <v>10</v>
+      </c>
+      <c r="G2">
+        <v>0</v>
+      </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A3" s="1" t="s">
         <v>6</v>
       </c>
@@ -2056,8 +2606,14 @@
       <c r="D3">
         <v>2.6649325265323101</v>
       </c>
+      <c r="F3" t="s">
+        <v>6</v>
+      </c>
+      <c r="G3">
+        <v>1.41730194714546</v>
+      </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A4" s="1" t="s">
         <v>8</v>
       </c>
@@ -2070,8 +2626,14 @@
       <c r="D4">
         <v>2.5977483063393199</v>
       </c>
+      <c r="F4" t="s">
+        <v>12</v>
+      </c>
+      <c r="G4">
+        <v>1.4176127011742199</v>
+      </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A5" s="1" t="s">
         <v>10</v>
       </c>
@@ -2084,8 +2646,14 @@
       <c r="D5">
         <v>2.54076374062651</v>
       </c>
+      <c r="F5" t="s">
+        <v>10</v>
+      </c>
+      <c r="G5">
+        <v>0</v>
+      </c>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A6" s="1" t="s">
         <v>12</v>
       </c>
@@ -2098,8 +2666,14 @@
       <c r="D6">
         <v>2.5876237612164901</v>
       </c>
+      <c r="F6" t="s">
+        <v>20</v>
+      </c>
+      <c r="G6">
+        <v>1.2780348272281099</v>
+      </c>
     </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A7" s="1" t="s">
         <v>14</v>
       </c>
@@ -2112,8 +2686,14 @@
       <c r="D7">
         <v>1.83320161865776</v>
       </c>
+      <c r="F7" t="s">
+        <v>14</v>
+      </c>
+      <c r="G7">
+        <v>0.88988790262010298</v>
+      </c>
     </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A8" s="1" t="s">
         <v>16</v>
       </c>
@@ -2126,8 +2706,14 @@
       <c r="D8">
         <v>3.09235839203461</v>
       </c>
+      <c r="F8" t="s">
+        <v>16</v>
+      </c>
+      <c r="G8">
+        <v>2.7341953492741502</v>
+      </c>
     </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A9" s="1" t="s">
         <v>18</v>
       </c>
@@ -2139,6 +2725,12 @@
       </c>
       <c r="D9">
         <v>2.4915844109666501</v>
+      </c>
+      <c r="F9" t="s">
+        <v>4</v>
+      </c>
+      <c r="G9">
+        <v>1.4755046936425</v>
       </c>
     </row>
   </sheetData>

</xml_diff>